<commit_message>
Added R0A config with 320 MHz on all outputs from 48 MHz crystal
</commit_message>
<xml_diff>
--- a/ClockBuilderPRO/test_projects/TestConfigurationIndex.xlsx
+++ b/ClockBuilderPRO/test_projects/TestConfigurationIndex.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\6089-127_CM_V3\GitHub\Cornell_CM_Rev3_HW\ClockBuilderPRO\test_projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\6089-127_CM_V3\GitHub\ClockBuilderPRO\test_projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB3D9E2-94B1-4B26-AD3F-D321C11F063A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C851E73D-8468-4176-9109-48A9C99D14C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{317829E7-0442-4B0F-847B-BF9A16B0382F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="185">
   <si>
     <t>Common</t>
   </si>
@@ -590,6 +590,9 @@
   </si>
   <si>
     <t>R0Bv3X05</t>
+  </si>
+  <si>
+    <t>R0Av3X03</t>
   </si>
 </sst>
 </file>
@@ -1092,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AAA10E1-D638-4109-9638-B5E913BD74DD}">
-  <dimension ref="A1:S59"/>
+  <dimension ref="A1:S60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
@@ -1260,77 +1263,80 @@
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="S11" s="4"/>
+      <c r="A11" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="12">
+        <v>48</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="I11" s="11">
+        <v>320</v>
+      </c>
+      <c r="J11" s="11">
+        <v>320</v>
+      </c>
+      <c r="K11" s="11">
+        <v>320</v>
+      </c>
+      <c r="L11" s="11">
+        <v>320</v>
+      </c>
+      <c r="M11" s="11">
+        <v>320</v>
+      </c>
+      <c r="N11" s="11">
+        <v>320</v>
+      </c>
+      <c r="O11" s="11">
+        <v>320</v>
+      </c>
+      <c r="P11" s="11">
+        <v>320</v>
+      </c>
+      <c r="Q11" s="11">
+        <v>320</v>
+      </c>
+      <c r="R11" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="S11" s="13" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="5">
-        <v>48</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I12" s="1">
-        <v>310</v>
-      </c>
-      <c r="J12" s="1">
-        <v>155</v>
-      </c>
-      <c r="K12" s="1">
-        <v>290</v>
-      </c>
-      <c r="L12" s="1">
-        <v>145</v>
-      </c>
-      <c r="M12" s="1">
-        <v>270</v>
-      </c>
-      <c r="N12" s="1">
-        <v>135</v>
-      </c>
-      <c r="O12" s="1">
-        <v>250</v>
-      </c>
-      <c r="P12" s="1">
-        <v>125</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>230</v>
-      </c>
-      <c r="R12" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="S12" s="4"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>171</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="5">
-        <v>240</v>
+      <c r="C13" s="5">
+        <v>48</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>1</v>
@@ -1338,105 +1344,105 @@
       <c r="F13" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G13" s="5">
-        <v>240</v>
+      <c r="G13" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="I13" s="1">
-        <v>240</v>
+        <v>310</v>
       </c>
       <c r="J13" s="1">
-        <v>240</v>
+        <v>155</v>
       </c>
       <c r="K13" s="1">
-        <v>240</v>
+        <v>290</v>
       </c>
       <c r="L13" s="1">
-        <v>240</v>
+        <v>145</v>
       </c>
       <c r="M13" s="1">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="N13" s="1">
-        <v>240</v>
+        <v>135</v>
       </c>
       <c r="O13" s="1">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="P13" s="1">
-        <v>240</v>
+        <v>125</v>
       </c>
       <c r="Q13" s="1">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="R13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="S13" s="4">
-        <v>240</v>
+      <c r="S13" s="4" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E14" s="5">
-        <v>320</v>
+      <c r="D14" s="5">
+        <v>240</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G14" s="5">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="I14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="J14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="K14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="L14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="M14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="N14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="O14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="P14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="Q14" s="1">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="R14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="S14" s="4">
-        <v>320</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>0</v>
@@ -1444,180 +1450,180 @@
       <c r="D15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F15" s="5">
-        <v>40</v>
+      <c r="E15" s="5">
+        <v>320</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="G15" s="5">
-        <v>40</v>
+        <v>320</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="I15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="J15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="K15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="L15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="M15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="N15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="O15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="P15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="Q15" s="1">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="R15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="S15" s="4">
-        <v>40</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D16" s="5">
-        <v>240</v>
-      </c>
-      <c r="E16" s="5">
-        <v>320</v>
+      <c r="D16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="F16" s="5">
         <v>40</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>1</v>
+      <c r="G16" s="5">
+        <v>40</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="I16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="J16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="K16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="L16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="M16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="N16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="O16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="P16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="Q16" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="R16" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="S16" s="1" t="s">
-        <v>1</v>
+      <c r="S16" s="4">
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="S17" s="4"/>
+      <c r="A17" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <v>240</v>
+      </c>
+      <c r="E17" s="5">
+        <v>320</v>
+      </c>
+      <c r="F17" s="5">
+        <v>40</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I17" s="1">
+        <v>280</v>
+      </c>
+      <c r="J17" s="1">
+        <v>280</v>
+      </c>
+      <c r="K17" s="1">
+        <v>280</v>
+      </c>
+      <c r="L17" s="1">
+        <v>280</v>
+      </c>
+      <c r="M17" s="1">
+        <v>280</v>
+      </c>
+      <c r="N17" s="1">
+        <v>280</v>
+      </c>
+      <c r="O17" s="1">
+        <v>280</v>
+      </c>
+      <c r="P17" s="1">
+        <v>280</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>280</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="S17" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C18" s="5">
-        <v>48</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H18" s="1">
-        <v>60</v>
-      </c>
-      <c r="I18" s="1">
-        <v>40</v>
-      </c>
-      <c r="J18" s="1">
-        <v>100</v>
-      </c>
-      <c r="K18" s="1">
-        <v>120</v>
-      </c>
-      <c r="L18" s="1">
-        <v>312</v>
-      </c>
-      <c r="M18" s="1">
-        <v>168</v>
-      </c>
-      <c r="N18" s="1">
-        <v>336</v>
-      </c>
-      <c r="O18" s="1">
-        <v>156</v>
-      </c>
-      <c r="P18" s="1">
-        <v>272</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>136</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A18" s="3"/>
+      <c r="S18" s="4"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>175</v>
+        <v>33</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="5">
-        <v>320</v>
+      <c r="C19" s="5">
+        <v>48</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>1</v>
@@ -1625,105 +1631,105 @@
       <c r="F19" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G19" s="5">
-        <v>320</v>
+      <c r="G19" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="H19" s="1">
-        <v>320</v>
+        <v>60</v>
       </c>
       <c r="I19" s="1">
-        <v>320</v>
+        <v>40</v>
       </c>
       <c r="J19" s="1">
-        <v>320</v>
+        <v>100</v>
       </c>
       <c r="K19" s="1">
-        <v>320</v>
+        <v>120</v>
       </c>
       <c r="L19" s="1">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="M19" s="1">
-        <v>320</v>
+        <v>168</v>
       </c>
       <c r="N19" s="1">
-        <v>320</v>
+        <v>336</v>
       </c>
       <c r="O19" s="1">
-        <v>320</v>
+        <v>156</v>
       </c>
       <c r="P19" s="1">
-        <v>320</v>
+        <v>272</v>
       </c>
       <c r="Q19" s="1">
-        <v>320</v>
+        <v>136</v>
       </c>
       <c r="R19" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="S19" s="4">
-        <v>320</v>
+      <c r="S19" s="4" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E20" s="5">
-        <v>40</v>
+      <c r="D20" s="5">
+        <v>320</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G20" s="5">
-        <v>40</v>
+        <v>320</v>
       </c>
       <c r="H20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="I20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="J20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="K20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="L20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="M20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="N20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="O20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="P20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="Q20" s="1">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="R20" s="1" t="s">
         <v>2</v>
       </c>
       <c r="S20" s="4">
-        <v>40</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>0</v>
@@ -1731,44 +1737,44 @@
       <c r="D21" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F21" s="5">
+      <c r="E21" s="5">
         <v>40</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="G21" s="5">
         <v>40</v>
       </c>
       <c r="H21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="I21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="J21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="K21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="L21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="M21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="N21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="O21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="P21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="Q21" s="1">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="R21" s="1" t="s">
         <v>2</v>
@@ -1778,77 +1784,77 @@
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="S22" s="4"/>
+      <c r="A22" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F22" s="5">
+        <v>40</v>
+      </c>
+      <c r="G22" s="5">
+        <v>40</v>
+      </c>
+      <c r="H22" s="1">
+        <v>120</v>
+      </c>
+      <c r="I22" s="1">
+        <v>120</v>
+      </c>
+      <c r="J22" s="1">
+        <v>120</v>
+      </c>
+      <c r="K22" s="1">
+        <v>120</v>
+      </c>
+      <c r="L22" s="1">
+        <v>120</v>
+      </c>
+      <c r="M22" s="1">
+        <v>120</v>
+      </c>
+      <c r="N22" s="1">
+        <v>120</v>
+      </c>
+      <c r="O22" s="1">
+        <v>120</v>
+      </c>
+      <c r="P22" s="1">
+        <v>120</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>120</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="S22" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" s="5">
-        <v>48</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H23" s="1">
-        <v>176</v>
-      </c>
-      <c r="I23" s="1">
-        <v>220</v>
-      </c>
-      <c r="J23" s="1">
-        <v>110</v>
-      </c>
-      <c r="K23" s="1">
-        <v>132</v>
-      </c>
-      <c r="L23" s="1">
-        <v>296</v>
-      </c>
-      <c r="M23" s="1">
-        <v>163</v>
-      </c>
-      <c r="N23" s="1">
-        <v>326</v>
-      </c>
-      <c r="O23" s="1">
-        <v>148</v>
-      </c>
-      <c r="P23" s="1">
-        <v>268</v>
-      </c>
-      <c r="Q23" s="1">
-        <v>132</v>
-      </c>
-      <c r="R23" s="1">
-        <v>55</v>
-      </c>
-      <c r="S23" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="A23" s="3"/>
+      <c r="S23" s="4"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>178</v>
+        <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D24" s="5">
-        <v>100</v>
+      <c r="C24" s="5">
+        <v>48</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>1</v>
@@ -1856,105 +1862,105 @@
       <c r="F24" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G24" s="5">
-        <v>100</v>
+      <c r="G24" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="H24" s="1">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="I24" s="1">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="J24" s="1">
-        <v>200</v>
+        <v>110</v>
       </c>
       <c r="K24" s="1">
-        <v>200</v>
+        <v>132</v>
       </c>
       <c r="L24" s="1">
-        <v>200</v>
+        <v>296</v>
       </c>
       <c r="M24" s="1">
-        <v>200</v>
+        <v>163</v>
       </c>
       <c r="N24" s="1">
-        <v>200</v>
+        <v>326</v>
       </c>
       <c r="O24" s="1">
-        <v>200</v>
+        <v>148</v>
       </c>
       <c r="P24" s="1">
-        <v>200</v>
+        <v>268</v>
       </c>
       <c r="Q24" s="1">
-        <v>200</v>
+        <v>132</v>
       </c>
       <c r="R24" s="1">
-        <v>200</v>
-      </c>
-      <c r="S24" s="4">
-        <v>100</v>
+        <v>55</v>
+      </c>
+      <c r="S24" s="4" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E25" s="5">
-        <v>40</v>
+      <c r="D25" s="5">
+        <v>100</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G25" s="5">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="H25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="I25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="J25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="K25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="L25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="M25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="N25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="O25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="P25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="Q25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="R25" s="1">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="S25" s="4">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>0</v>
@@ -1962,127 +1968,127 @@
       <c r="D26" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F26" s="5">
+      <c r="E26" s="5">
         <v>40</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="G26" s="5">
         <v>40</v>
       </c>
       <c r="H26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="I26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="J26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="K26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="L26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="M26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="N26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="O26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="P26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="Q26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="R26" s="1">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="S26" s="4">
         <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="S27" s="4"/>
+      <c r="A27" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F27" s="5">
+        <v>40</v>
+      </c>
+      <c r="G27" s="5">
+        <v>40</v>
+      </c>
+      <c r="H27" s="1">
+        <v>140</v>
+      </c>
+      <c r="I27" s="1">
+        <v>140</v>
+      </c>
+      <c r="J27" s="1">
+        <v>140</v>
+      </c>
+      <c r="K27" s="1">
+        <v>140</v>
+      </c>
+      <c r="L27" s="1">
+        <v>140</v>
+      </c>
+      <c r="M27" s="1">
+        <v>140</v>
+      </c>
+      <c r="N27" s="1">
+        <v>140</v>
+      </c>
+      <c r="O27" s="1">
+        <v>140</v>
+      </c>
+      <c r="P27" s="1">
+        <v>140</v>
+      </c>
+      <c r="Q27" s="1">
+        <v>140</v>
+      </c>
+      <c r="R27" s="1">
+        <v>140</v>
+      </c>
+      <c r="S27" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C28" s="5">
-        <v>48</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H28" s="1">
-        <v>116</v>
-      </c>
-      <c r="I28" s="1">
-        <v>232</v>
-      </c>
-      <c r="J28" s="1">
-        <v>174</v>
-      </c>
-      <c r="K28" s="1">
-        <v>348</v>
-      </c>
-      <c r="L28" s="1">
-        <v>310</v>
-      </c>
-      <c r="M28" s="1">
-        <v>170</v>
-      </c>
-      <c r="N28" s="1">
-        <v>340</v>
-      </c>
-      <c r="O28" s="1">
-        <v>155</v>
-      </c>
-      <c r="P28" s="1">
-        <v>286</v>
-      </c>
-      <c r="Q28" s="1">
-        <v>143</v>
-      </c>
-      <c r="R28" s="1">
-        <v>226</v>
-      </c>
-      <c r="S28" s="4">
-        <v>113</v>
-      </c>
+      <c r="A28" s="3"/>
+      <c r="S28" s="4"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>181</v>
+        <v>35</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D29" s="5">
-        <v>120</v>
+      <c r="C29" s="5">
+        <v>48</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>1</v>
@@ -2091,104 +2097,157 @@
         <v>2</v>
       </c>
       <c r="H29" s="1">
+        <v>116</v>
+      </c>
+      <c r="I29" s="1">
+        <v>232</v>
+      </c>
+      <c r="J29" s="1">
+        <v>174</v>
+      </c>
+      <c r="K29" s="1">
+        <v>348</v>
+      </c>
+      <c r="L29" s="1">
+        <v>310</v>
+      </c>
+      <c r="M29" s="1">
+        <v>170</v>
+      </c>
+      <c r="N29" s="1">
+        <v>340</v>
+      </c>
+      <c r="O29" s="1">
+        <v>155</v>
+      </c>
+      <c r="P29" s="1">
+        <v>286</v>
+      </c>
+      <c r="Q29" s="1">
+        <v>143</v>
+      </c>
+      <c r="R29" s="1">
+        <v>226</v>
+      </c>
+      <c r="S29" s="4">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5">
+        <v>120</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H30" s="1">
         <v>240</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I30" s="1">
         <v>240</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J30" s="1">
         <v>240</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K30" s="1">
         <v>240</v>
       </c>
-      <c r="L29" s="1">
+      <c r="L30" s="1">
         <v>240</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M30" s="1">
         <v>240</v>
       </c>
-      <c r="N29" s="1">
+      <c r="N30" s="1">
         <v>240</v>
       </c>
-      <c r="O29" s="1">
+      <c r="O30" s="1">
         <v>240</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P30" s="1">
         <v>240</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q30" s="1">
         <v>240</v>
       </c>
-      <c r="R29" s="1">
+      <c r="R30" s="1">
         <v>240</v>
       </c>
-      <c r="S29" s="4">
+      <c r="S30" s="4">
         <v>240</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B31" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="F30" s="8">
+      <c r="C31" s="7"/>
+      <c r="D31" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="F31" s="8">
         <v>40</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G31" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H31" s="7">
         <v>180</v>
       </c>
-      <c r="I30" s="7">
+      <c r="I31" s="7">
         <v>180</v>
       </c>
-      <c r="J30" s="7">
+      <c r="J31" s="7">
         <v>180</v>
       </c>
-      <c r="K30" s="7">
+      <c r="K31" s="7">
         <v>180</v>
       </c>
-      <c r="L30" s="7">
+      <c r="L31" s="7">
         <v>180</v>
       </c>
-      <c r="M30" s="7">
+      <c r="M31" s="7">
         <v>180</v>
       </c>
-      <c r="N30" s="7">
+      <c r="N31" s="7">
         <v>180</v>
       </c>
-      <c r="O30" s="7">
+      <c r="O31" s="7">
         <v>180</v>
       </c>
-      <c r="P30" s="7">
+      <c r="P31" s="7">
         <v>180</v>
       </c>
-      <c r="Q30" s="7">
+      <c r="Q31" s="7">
         <v>180</v>
       </c>
-      <c r="R30" s="7">
+      <c r="R31" s="7">
         <v>180</v>
       </c>
-      <c r="S30" s="9">
+      <c r="S31" s="9">
         <v>180</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="S31" s="1"/>
-    </row>
-    <row r="40" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S40" s="1"/>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S32" s="1"/>
     </row>
     <row r="41" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S41" s="1"/>
@@ -2196,8 +2255,8 @@
     <row r="42" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S42" s="1"/>
     </row>
-    <row r="44" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S44" s="1"/>
+    <row r="43" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S43" s="1"/>
     </row>
     <row r="45" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S45" s="1"/>
@@ -2211,8 +2270,8 @@
     <row r="48" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S48" s="1"/>
     </row>
-    <row r="50" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S50" s="1"/>
+    <row r="49" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S49" s="1"/>
     </row>
     <row r="51" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S51" s="1"/>
@@ -2229,14 +2288,17 @@
     <row r="55" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S55" s="1"/>
     </row>
-    <row r="57" spans="19:19" x14ac:dyDescent="0.25">
-      <c r="S57" s="1"/>
+    <row r="56" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S56" s="1"/>
     </row>
     <row r="58" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S58" s="1"/>
     </row>
     <row r="59" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S59" s="1"/>
+    </row>
+    <row r="60" spans="19:19" x14ac:dyDescent="0.25">
+      <c r="S60" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated config file database
</commit_message>
<xml_diff>
--- a/ClockBuilderPRO/test_projects/TestConfigurationIndex.xlsx
+++ b/ClockBuilderPRO/test_projects/TestConfigurationIndex.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\6089-127_CM_V3\GitHub\ClockBuilderPRO\test_projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C851E73D-8468-4176-9109-48A9C99D14C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57402D53-4BA2-4D37-8184-A7DAD32F19C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{317829E7-0442-4B0F-847B-BF9A16B0382F}"/>
   </bookViews>
@@ -1288,31 +1288,31 @@
         <v>2</v>
       </c>
       <c r="I11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="J11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="K11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="L11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="M11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="N11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="O11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="P11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="Q11" s="11">
-        <v>320</v>
+        <v>320.63</v>
       </c>
       <c r="R11" s="11" t="s">
         <v>2</v>

</xml_diff>